<commit_message>
daily-jobs: biostat SM/AD scrape for 2026-10-20
</commit_message>
<xml_diff>
--- a/daily-jobs/manual-check-latest.xlsx
+++ b/daily-jobs/manual-check-latest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Manual check 2026-10-19" sheetId="1" r:id="rId1"/>
+    <sheet name="Manual check 2026-10-20" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -583,7 +583,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 422 Unprocessable Entity</t>
+          <t xml:space="preserve">HTTP 520 &lt;none&gt;</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">

</xml_diff>

<commit_message>
daily-jobs: biostat SM/AD scrape for 2026-10-21
</commit_message>
<xml_diff>
--- a/daily-jobs/manual-check-latest.xlsx
+++ b/daily-jobs/manual-check-latest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Manual check 2026-10-20" sheetId="1" r:id="rId1"/>
+    <sheet name="Manual check 2026-10-21" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -583,7 +583,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTTP 520 &lt;none&gt;</t>
+          <t xml:space="preserve">HTTP 422 Unprocessable Entity</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">

</xml_diff>

<commit_message>
daily-jobs: biostat SM/AD scrape for 2026-10-26
</commit_message>
<xml_diff>
--- a/daily-jobs/manual-check-latest.xlsx
+++ b/daily-jobs/manual-check-latest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Manual check 2026-10-25" sheetId="1" r:id="rId1"/>
+    <sheet name="Manual check 2026-10-26" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -1895,7 +1895,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">scanned=0 title_hits=0 in_24h=0 (0.1s)</t>
+          <t xml:space="preserve">scanned=0 title_hits=0 in_24h=0 (0.2s)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">

</xml_diff>